<commit_message>
Kit Medicos: 41 prompts na pagina, copy, oferta, e-mails e textos de anuncio; 156 pacientes na oferta; planilha 14 sem boleto
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0146uBo6FVJ2cyEehyP8rK61
</commit_message>
<xml_diff>
--- a/projetos/gestao-ia-planilhas/produto/kit-medicos/14-parcelas-e-inadimplencia.xlsx
+++ b/projetos/gestao-ia-planilhas/produto/kit-medicos/14-parcelas-e-inadimplencia.xlsx
@@ -1209,7 +1209,7 @@
       </c>
       <c r="E11" s="27" t="str">
         <f>IF(Config!$C$10="","",Config!$B$10)</f>
-        <v>Lembrete gentil por WhatsApp: confirmar se o Pix ou o boleto chegou e reenviar, se preciso.</v>
+        <v>Lembrete gentil por WhatsApp: confirmar se o Pix chegou e reenviar o link de pagamento, se preciso.</v>
       </c>
       <c r="F11" s="21" t="n"/>
       <c r="G11" s="21" t="n"/>
@@ -2229,7 +2229,7 @@
       </c>
       <c r="B10" s="36" t="inlineStr">
         <is>
-          <t>Lembrete gentil por WhatsApp: confirmar se o Pix ou o boleto chegou e reenviar, se preciso.</t>
+          <t>Lembrete gentil por WhatsApp: confirmar se o Pix chegou e reenviar o link de pagamento, se preciso.</t>
         </is>
       </c>
       <c r="C10" s="24" t="str">
@@ -22212,7 +22212,7 @@
       </c>
       <c r="M138" s="23" t="str">
         <f>IF(I138&lt;&gt;"Vencida","",IF(COUNTIF(Config!$A$10:$A$13,"&lt;="&amp;J138)=0,"Aguardar: ainda não chegou ao primeiro passo da régua.",INDEX(Config!$B$10:$B$13,COUNTIF(Config!$A$10:$A$13,"&lt;="&amp;J138))))</f>
-        <v>Lembrete gentil por WhatsApp: confirmar se o Pix ou o boleto chegou e reenviar, se preciso.</v>
+        <v>Lembrete gentil por WhatsApp: confirmar se o Pix chegou e reenviar o link de pagamento, se preciso.</v>
       </c>
       <c r="N138" s="39">
         <f>IF(I138="Vencida",F138*J138+ROW()/100000,0)</f>
@@ -23346,7 +23346,7 @@
       </c>
       <c r="M157" s="23" t="str">
         <f>IF(I157&lt;&gt;"Vencida","",IF(COUNTIF(Config!$A$10:$A$13,"&lt;="&amp;J157)=0,"Aguardar: ainda não chegou ao primeiro passo da régua.",INDEX(Config!$B$10:$B$13,COUNTIF(Config!$A$10:$A$13,"&lt;="&amp;J157))))</f>
-        <v>Lembrete gentil por WhatsApp: confirmar se o Pix ou o boleto chegou e reenviar, se preciso.</v>
+        <v>Lembrete gentil por WhatsApp: confirmar se o Pix chegou e reenviar o link de pagamento, se preciso.</v>
       </c>
       <c r="N157" s="39">
         <f>IF(I157="Vencida",F157*J157+ROW()/100000,0)</f>

</xml_diff>